<commit_message>
feat(excel): PIMS-shaped Excel → mono+ADMM → results workbook MVP
End-to-end classic converter path for planners living in Excel:
- load Crudes/Products/Capacities template
- solve_simple_monolithic + package ADMM (qp_l2, recover_primal, ρ=15)
- write results xlsx (Summary/rates/shadows) + JSON

Also: fix excel roundtrip test to assert against live assay JSON
(not hard-coded API 39.6); regenerate crudes_template.xlsx from
current detailed assays. Demo: python -m demos.run_excel_pipeline_demo
</commit_message>
<xml_diff>
--- a/data/assays/crudes_template.xlsx
+++ b/data/assays/crudes_template.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,25 +498,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39.6</v>
+        <v>47.39987725648041</v>
       </c>
       <c r="C2" t="n">
-        <v>0.24</v>
+        <v>0.0698981115791165</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8</v>
+        <v>0.1185965915483614</v>
       </c>
       <c r="E2" t="n">
-        <v>900</v>
+        <v>113.3293611436626</v>
       </c>
       <c r="F2" t="n">
-        <v>0.42</v>
+        <v>0.4255761386139089</v>
       </c>
       <c r="G2" t="n">
-        <v>0.32</v>
+        <v>0.4479975255697073</v>
       </c>
       <c r="H2" t="n">
-        <v>0.26</v>
+        <v>0.1239958152669457</v>
       </c>
       <c r="I2" t="n">
         <v>78</v>
@@ -525,16 +525,16 @@
         <v>100</v>
       </c>
       <c r="K2" t="n">
-        <v>0.28</v>
+        <v>0.503</v>
       </c>
       <c r="L2" t="n">
-        <v>0.3</v>
+        <v>0.297</v>
       </c>
       <c r="M2" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="N2" t="n">
-        <v>0.16</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="3">
@@ -544,25 +544,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>28.9</v>
+        <v>28.4</v>
       </c>
       <c r="C3" t="n">
-        <v>1.85</v>
+        <v>2.17</v>
       </c>
       <c r="D3" t="n">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="F3" t="n">
         <v>0.3</v>
       </c>
       <c r="G3" t="n">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="H3" t="n">
-        <v>0.36</v>
+        <v>0.4</v>
       </c>
       <c r="I3" t="n">
         <v>72</v>
@@ -571,16 +571,16 @@
         <v>80</v>
       </c>
       <c r="K3" t="n">
-        <v>0.18</v>
+        <v>0.194</v>
       </c>
       <c r="L3" t="n">
-        <v>0.27</v>
+        <v>0.278</v>
       </c>
       <c r="M3" t="n">
-        <v>0.3</v>
+        <v>0.236</v>
       </c>
       <c r="N3" t="n">
-        <v>0.25</v>
+        <v>0.292</v>
       </c>
     </row>
     <row r="4">
@@ -678,47 +678,185 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Arab_Medium</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>68</v>
+      </c>
+      <c r="J6" t="n">
+        <v>80</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.288</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Bonny_Light</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B7" t="n">
         <v>35.5</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C7" t="n">
         <v>0.16</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>1.1</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E7" t="n">
         <v>700</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F7" t="n">
         <v>0.45</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G7" t="n">
         <v>0.33</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H7" t="n">
         <v>0.22</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I7" t="n">
         <v>80</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J7" t="n">
         <v>70</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K7" t="n">
         <v>0.26</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L7" t="n">
         <v>0.32</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M7" t="n">
         <v>0.25</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N7" t="n">
         <v>0.17</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cold_Lake_Blend</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3062</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.217</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.631</v>
+      </c>
+      <c r="I8" t="n">
+        <v>58</v>
+      </c>
+      <c r="J8" t="n">
+        <v>50</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.301</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.324</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Basrah_Medium</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>68</v>
+      </c>
+      <c r="J9" t="n">
+        <v>80</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>